<commit_message>
Fix thighs results: add muscle labels
</commit_message>
<xml_diff>
--- a/get_results/results/vol.2_dixon3pt_t2slice/results.xlsx
+++ b/get_results/results/vol.2_dixon3pt_t2slice/results.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -509,7 +509,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -542,7 +542,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -575,7 +575,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -674,7 +674,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -707,7 +707,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -740,7 +740,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -773,7 +773,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -806,7 +806,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -872,7 +872,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -905,7 +905,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -938,7 +938,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -971,7 +971,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -4135,7 +4135,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -5102,7 +5102,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -5918,7 +5918,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5992,7 +5992,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -6097,7 +6097,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -6134,7 +6134,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -6350,7 +6350,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -6424,7 +6424,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -6461,7 +6461,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -6566,7 +6566,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D206" t="n">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D208" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -7368,7 +7368,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D217" t="n">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D218" t="n">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D220" t="n">
@@ -7615,7 +7615,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -7868,7 +7868,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D228" t="n">
@@ -7905,7 +7905,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D229" t="n">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D230" t="n">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D231" t="n">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -8047,7 +8047,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -8232,7 +8232,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -8263,7 +8263,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -8300,7 +8300,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -8337,7 +8337,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -8448,7 +8448,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -8485,7 +8485,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -8522,7 +8522,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -8590,7 +8590,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -8627,7 +8627,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -8701,7 +8701,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -8843,7 +8843,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -8880,7 +8880,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -8917,7 +8917,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -9065,7 +9065,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -9170,7 +9170,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -9281,7 +9281,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -9423,7 +9423,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D272" t="n">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -9534,7 +9534,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D275" t="n">
@@ -9608,7 +9608,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D276" t="n">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D277" t="n">
@@ -9682,7 +9682,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -9713,7 +9713,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -9750,7 +9750,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -9787,7 +9787,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D284" t="n">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D285" t="n">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -10040,7 +10040,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D288" t="n">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>LABEL_1</t>
+          <t>TA_R</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -10145,7 +10145,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>LABEL_2</t>
+          <t>ED_R</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>LABEL_3</t>
+          <t>PER_R</t>
         </is>
       </c>
       <c r="D292" t="n">
@@ -10219,7 +10219,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>LABEL_4</t>
+          <t>DLPC_R</t>
         </is>
       </c>
       <c r="D293" t="n">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>LABEL_5</t>
+          <t>POP_R</t>
         </is>
       </c>
       <c r="D294" t="n">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>LABEL_6</t>
+          <t>SOL_R</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -10330,7 +10330,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>LABEL_7</t>
+          <t>GAS_MED_R</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -10367,7 +10367,7 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>LABEL_8</t>
+          <t>GAS_LAT_R</t>
         </is>
       </c>
       <c r="D297" t="n">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>LABEL_9</t>
+          <t>TA_L</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -10441,7 +10441,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>LABEL_10</t>
+          <t>ED_L</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>LABEL_11</t>
+          <t>PER_L</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -10515,7 +10515,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>LABEL_12</t>
+          <t>DLPC_L</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -10552,7 +10552,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>LABEL_13</t>
+          <t>POP_L</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -10589,7 +10589,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>LABEL_14</t>
+          <t>SOL_L</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -10626,7 +10626,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>LABEL_15</t>
+          <t>GAS_MED_L</t>
         </is>
       </c>
       <c r="D304" t="n">
@@ -10663,7 +10663,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>LABEL_16</t>
+          <t>GAS_LAT_L</t>
         </is>
       </c>
       <c r="D305" t="n">

</xml_diff>